<commit_message>
set up analysis for TECH_XG_009,, Tile 1 only first two time points have images , rest is empty
</commit_message>
<xml_diff>
--- a/Experiments/TECH_XG_009/setup.xlsx
+++ b/Experiments/TECH_XG_009/setup.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="33">
   <si>
     <t>Key</t>
   </si>
@@ -72,13 +72,13 @@
     <t>path</t>
   </si>
   <si>
-    <t>HFE7500_K562_droplets_300mbaroil_150mbar</t>
-  </si>
-  <si>
-    <t>/Users/xiangxigao/Desktop/DMi8/TECH_XG_006/TECH_XG_006.lif</t>
-  </si>
-  <si>
-    <t>RAN101_K562_droplets_300mbaroil_150mbar</t>
+    <t>HFE7500_THP1_300_170</t>
+  </si>
+  <si>
+    <t>/Users/xiangxigao/Desktop/DMi8/TECH_XG_009/TECH_XG_009.lif</t>
+  </si>
+  <si>
+    <t>RAN101_THP1_300_170</t>
   </si>
   <si>
     <t>channel_index</t>
@@ -557,7 +557,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36.142857142857146" customWidth="1"/>
-    <col min="2" max="2" width="45.42857142857143" customWidth="1"/>
+    <col min="2" max="2" width="42.142857142857146" customWidth="1"/>
     <col min="3" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
@@ -641,15 +641,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
     <col min="2" max="3" width="15.285714285714286" customWidth="1"/>
     <col min="4" max="4" width="12.571428571428571" customWidth="1"/>
     <col min="5" max="6" width="13.571428571428571" customWidth="1"/>
-    <col min="7" max="7" width="49.714285714285715" customWidth="1"/>
-    <col min="8" max="8" width="58.57142857142857" customWidth="1"/>
+    <col min="7" max="7" width="29.428571428571427" customWidth="1"/>
+    <col min="8" max="8" width="77.28571428571429" customWidth="1"/>
     <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
@@ -690,7 +690,7 @@
         <v>5</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -716,10 +716,10 @@
         <v>5</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -742,10 +742,10 @@
         <v>5</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -768,10 +768,10 @@
         <v>5</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>4</v>
@@ -794,10 +794,10 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -820,10 +820,10 @@
         <v>5</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -846,10 +846,10 @@
         <v>5</v>
       </c>
       <c r="D8">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8">
         <v>7</v>
@@ -872,16 +872,16 @@
         <v>5</v>
       </c>
       <c r="D9">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>20</v>
@@ -898,16 +898,16 @@
         <v>5</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>20</v>
@@ -924,16 +924,16 @@
         <v>5</v>
       </c>
       <c r="D11">
+        <v>25</v>
+      </c>
+      <c r="E11">
         <v>7</v>
       </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
       <c r="F11">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>20</v>
@@ -950,16 +950,16 @@
         <v>5</v>
       </c>
       <c r="D12">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>20</v>
@@ -976,16 +976,16 @@
         <v>5</v>
       </c>
       <c r="D13">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>20</v>
@@ -1002,13 +1002,13 @@
         <v>5</v>
       </c>
       <c r="D14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G14" t="s">
         <v>21</v>
@@ -1028,13 +1028,13 @@
         <v>5</v>
       </c>
       <c r="D15">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G15" t="s">
         <v>21</v>
@@ -1044,32 +1044,264 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="H16" s="5"/>
+      <c r="A16" s="4">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>90</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>27</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>3</v>
+      </c>
+      <c r="G16" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
-      <c r="H17" s="5"/>
+      <c r="A17" s="4">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>90</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>28</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>4</v>
+      </c>
+      <c r="G17" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="4"/>
-      <c r="H18" s="5"/>
+      <c r="A18" s="4">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>90</v>
+      </c>
+      <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <v>29</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>5</v>
+      </c>
+      <c r="G18" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="H19" s="5"/>
+      <c r="A19" s="4">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>90</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>30</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>6</v>
+      </c>
+      <c r="G19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="H20" s="5"/>
+      <c r="A20" s="4">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>90</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>31</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
+        <v>7</v>
+      </c>
+      <c r="G20" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-      <c r="H21" s="5"/>
+      <c r="A21" s="4">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>90</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21">
+        <v>32</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <v>8</v>
+      </c>
+      <c r="G21" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
-      <c r="H22" s="5"/>
+      <c r="A22" s="4">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>90</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>33</v>
+      </c>
+      <c r="E22">
+        <v>6</v>
+      </c>
+      <c r="F22">
+        <v>9</v>
+      </c>
+      <c r="G22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>90</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <v>34</v>
+      </c>
+      <c r="E23">
+        <v>7</v>
+      </c>
+      <c r="F23">
+        <v>10</v>
+      </c>
+      <c r="G23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>90</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>35</v>
+      </c>
+      <c r="E24">
+        <v>8</v>
+      </c>
+      <c r="F24">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>90</v>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25">
+        <v>37</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
analysis of TECH_XG_009 THP1 cells in HFE7500 RAN101
</commit_message>
<xml_diff>
--- a/Experiments/TECH_XG_009/setup.xlsx
+++ b/Experiments/TECH_XG_009/setup.xlsx
@@ -649,7 +649,7 @@
     <col min="4" max="4" width="12.571428571428571" customWidth="1"/>
     <col min="5" max="6" width="13.571428571428571" customWidth="1"/>
     <col min="7" max="7" width="29.428571428571427" customWidth="1"/>
-    <col min="8" max="8" width="77.28571428571429" customWidth="1"/>
+    <col min="8" max="8" width="42.142857142857146" customWidth="1"/>
     <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
@@ -716,7 +716,7 @@
         <v>5</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -742,7 +742,7 @@
         <v>5</v>
       </c>
       <c r="D4">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -768,7 +768,7 @@
         <v>5</v>
       </c>
       <c r="D5">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -794,7 +794,7 @@
         <v>5</v>
       </c>
       <c r="D6">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E6">
         <v>2</v>
@@ -820,7 +820,7 @@
         <v>5</v>
       </c>
       <c r="D7">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -846,7 +846,7 @@
         <v>5</v>
       </c>
       <c r="D8">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -872,7 +872,7 @@
         <v>5</v>
       </c>
       <c r="D9">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -898,7 +898,7 @@
         <v>5</v>
       </c>
       <c r="D10">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E10">
         <v>6</v>
@@ -924,7 +924,7 @@
         <v>5</v>
       </c>
       <c r="D11">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E11">
         <v>7</v>
@@ -950,7 +950,7 @@
         <v>5</v>
       </c>
       <c r="D12">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E12">
         <v>8</v>
@@ -976,7 +976,7 @@
         <v>5</v>
       </c>
       <c r="D13">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1002,7 +1002,7 @@
         <v>5</v>
       </c>
       <c r="D14">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -1028,7 +1028,7 @@
         <v>5</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1054,7 +1054,7 @@
         <v>5</v>
       </c>
       <c r="D16">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -1080,7 +1080,7 @@
         <v>5</v>
       </c>
       <c r="D17">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -1106,7 +1106,7 @@
         <v>5</v>
       </c>
       <c r="D18">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -1132,7 +1132,7 @@
         <v>5</v>
       </c>
       <c r="D19">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E19">
         <v>3</v>
@@ -1158,7 +1158,7 @@
         <v>5</v>
       </c>
       <c r="D20">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="E20">
         <v>4</v>
@@ -1184,7 +1184,7 @@
         <v>5</v>
       </c>
       <c r="D21">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="E21">
         <v>5</v>
@@ -1210,7 +1210,7 @@
         <v>5</v>
       </c>
       <c r="D22">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="E22">
         <v>6</v>
@@ -1236,7 +1236,7 @@
         <v>5</v>
       </c>
       <c r="D23">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="E23">
         <v>7</v>
@@ -1262,7 +1262,7 @@
         <v>5</v>
       </c>
       <c r="D24">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E24">
         <v>8</v>
@@ -1288,7 +1288,7 @@
         <v>5</v>
       </c>
       <c r="D25">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E25">
         <v>0</v>

</xml_diff>